<commit_message>
Added Exercise 2A docs
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\disco\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33EAEEFA-BBC9-4A94-B7E9-78467858F863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F99485-52BE-44BE-8E5E-3C251E116D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{D48F8DFA-1C58-4E6A-8B24-AEBED868B4C8}"/>
   </bookViews>
@@ -36,67 +36,90 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>August</t>
-  </si>
-  <si>
-    <t>September</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>February</t>
-  </si>
-  <si>
-    <t>March</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>July</t>
-  </si>
-  <si>
-    <t>October</t>
-  </si>
-  <si>
-    <t>November</t>
-  </si>
-  <si>
-    <t>December</t>
-  </si>
-  <si>
-    <t>Klarna Purchases Over Time</t>
-  </si>
-  <si>
-    <t>Month:</t>
-  </si>
-  <si>
-    <t>Year:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Was The Data Downloadable? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">In my observation with Klarna, I noticed that I was unable to download the data, but just clicking on the months listed, I was able to go ahead and see what was spent in each month from 2023 to 2026, even though some of the months for 2026 have not come just yet.  </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+  <si>
+    <t>Name of Data Source</t>
+  </si>
+  <si>
+    <t>Depth of Coverage</t>
+  </si>
+  <si>
+    <t>Klarna</t>
+  </si>
+  <si>
+    <t>Steps To Download</t>
+  </si>
+  <si>
+    <t>Download Format</t>
+  </si>
+  <si>
+    <t>Type of Information</t>
+  </si>
+  <si>
+    <t>Purchases</t>
+  </si>
+  <si>
+    <t>Downloadable</t>
+  </si>
+  <si>
+    <t>Adittional Notes</t>
+  </si>
+  <si>
+    <t>Dating back to the first purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unable to download. </t>
+  </si>
+  <si>
+    <t>Download format unavailable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The information that I obtained through the account was only obtained by accessing my account, tapping on insights, and scrolling backwards to the data gathered from then to now. </t>
+  </si>
+  <si>
+    <t>Account Creation</t>
+  </si>
+  <si>
+    <t>Tweets and Photos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes. </t>
+  </si>
+  <si>
+    <t>Twitter (Desktop Version)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start on homepage, click on "more", then navihgate to "settings and privacy", then navigate to "your account", and finally, click on "download an archive of your data". </t>
+  </si>
+  <si>
+    <t>Zip file</t>
+  </si>
+  <si>
+    <t>I am chronically online and it really shows in how much I access twitter within my daily life.</t>
+  </si>
+  <si>
+    <t>Tumblr (Desktop Version)</t>
+  </si>
+  <si>
+    <t>Posts, Photos, and Reblogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start on homepage, click on "settings", then navigate to "privacy", and finally click on "request pirvacy data". </t>
+  </si>
+  <si>
+    <t>Zip file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most of the information within the file was from two different blogs for two different reasons because I kept them organized in a way to keep two of my interests separate so I am not feeling crowded on just one singular blog. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -126,10 +149,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -467,239 +488,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B30E6B9-CC9E-49DA-8EDB-AFD76AC500E2}">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.1796875" customWidth="1"/>
-    <col min="2" max="2" width="39.81640625" customWidth="1"/>
-    <col min="10" max="10" width="9.453125" customWidth="1"/>
-    <col min="12" max="12" width="9.08984375" customWidth="1"/>
-    <col min="13" max="13" width="9.36328125" customWidth="1"/>
+    <col min="1" max="1" width="21.26953125" customWidth="1"/>
+    <col min="2" max="2" width="22.90625" customWidth="1"/>
+    <col min="3" max="3" width="15.81640625" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="144" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
-        <v>13</v>
+    <row r="3" spans="1:7" ht="157.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="4" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" t="s">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
-        <v>1</v>
-      </c>
-      <c r="K3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M3" t="s">
-        <v>11</v>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>2023</v>
-      </c>
-      <c r="B4" s="1">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1">
-        <v>0</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2">
-        <v>229.84</v>
-      </c>
-      <c r="J4" s="1">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2">
-        <v>72.08</v>
-      </c>
-      <c r="L4" s="2">
-        <v>401.91</v>
-      </c>
-      <c r="M4" s="2">
-        <v>198.31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>2024</v>
-      </c>
-      <c r="B5" s="1">
-        <v>680.99</v>
-      </c>
-      <c r="C5" s="1">
-        <v>55.06</v>
-      </c>
-      <c r="D5">
-        <v>1182.96</v>
-      </c>
-      <c r="E5" s="1">
-        <v>397.85</v>
-      </c>
-      <c r="F5" s="1">
-        <v>338.24</v>
-      </c>
-      <c r="G5" s="2">
-        <v>594.12</v>
-      </c>
-      <c r="H5" s="2">
-        <v>460.25</v>
-      </c>
-      <c r="I5" s="1">
-        <v>42.39</v>
-      </c>
-      <c r="J5" s="2">
-        <v>356.47</v>
-      </c>
-      <c r="K5" s="2">
-        <v>690.31</v>
-      </c>
-      <c r="L5" s="2">
-        <v>384.62</v>
-      </c>
-      <c r="M5" s="2">
-        <v>469.46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>2025</v>
-      </c>
-      <c r="B6" s="2">
-        <v>881.78</v>
-      </c>
-      <c r="C6" s="2">
-        <v>191.78</v>
-      </c>
-      <c r="D6" s="2">
-        <v>287.47000000000003</v>
-      </c>
-      <c r="E6" s="2">
-        <v>247</v>
-      </c>
-      <c r="F6" s="2">
-        <v>226.06</v>
-      </c>
-      <c r="G6" s="2">
-        <v>245.12</v>
-      </c>
-      <c r="H6" s="2">
-        <v>915.55</v>
-      </c>
-      <c r="I6" s="2">
-        <v>303.92</v>
-      </c>
-      <c r="J6" s="2">
-        <v>236.22</v>
-      </c>
-      <c r="K6" s="2">
-        <v>444.11</v>
-      </c>
-      <c r="L6" s="2">
-        <v>461.98</v>
-      </c>
-      <c r="M6" s="2">
-        <v>327.56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>2026</v>
-      </c>
-      <c r="B7" s="2">
-        <v>625.94000000000005</v>
-      </c>
-      <c r="C7" s="2">
-        <v>975.95</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0</v>
-      </c>
-      <c r="J7" s="1">
-        <v>0</v>
-      </c>
-      <c r="K7" s="1">
-        <v>0</v>
-      </c>
-      <c r="L7" s="1">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="84.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
+    <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>